<commit_message>
Added new items from streams.
</commit_message>
<xml_diff>
--- a/QMS/Logs/MDL‑005 Engineering Change Control Log.xlsx
+++ b/QMS/Logs/MDL‑005 Engineering Change Control Log.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="17">
   <si>
     <t xml:space="preserve">ECR and ECN Log</t>
   </si>
@@ -67,6 +67,28 @@
   <si>
     <t xml:space="preserve">ECN-P1012202501-01-17-26-01</t>
   </si>
+  <si>
+    <t xml:space="preserve">P1012202501-01-26-26-01</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ECN-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">P1012202501-01-26-26-01</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -76,7 +98,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -104,6 +126,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -161,7 +188,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -191,6 +218,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -591,19 +622,33 @@
       <c r="U7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="A8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="7" t="n">
+        <v>46048</v>
+      </c>
+      <c r="D8" s="7"/>
+      <c r="E8" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
+      <c r="G8" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
+      <c r="K8" s="7" t="n">
+        <v>46048</v>
+      </c>
+      <c r="L8" s="7"/>
+      <c r="M8" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>

</xml_diff>